<commit_message>
ci: refresh reports & README last-run summary (2026-09-13 07:06 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-12 06:48 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-12 06:48 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A358"/>
+  <dimension ref="A1:A359"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3440,6 +3440,13 @@
       <c r="A358" t="inlineStr">
         <is>
           <t>2026-09-12 06:48 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="359">
+      <c r="A359" t="inlineStr">
+        <is>
+          <t>2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3463,7 +3470,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-12 06:48 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3629,7 +3636,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-12 06:48 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3765,7 +3772,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-12 06:48 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-14 07:30 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A359"/>
+  <dimension ref="A1:A360"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3447,6 +3447,13 @@
       <c r="A359" t="inlineStr">
         <is>
           <t>2026-09-13 07:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="360">
+      <c r="A360" t="inlineStr">
+        <is>
+          <t>2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3470,7 +3477,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3636,7 +3643,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3772,7 +3779,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-13 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-15 07:07 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A360"/>
+  <dimension ref="A1:A361"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3454,6 +3454,13 @@
       <c r="A360" t="inlineStr">
         <is>
           <t>2026-09-14 07:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="361">
+      <c r="A361" t="inlineStr">
+        <is>
+          <t>2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3477,7 +3484,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3643,7 +3650,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3779,7 +3786,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-14 07:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-16 07:07 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A361"/>
+  <dimension ref="A1:A362"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3461,6 +3461,13 @@
       <c r="A361" t="inlineStr">
         <is>
           <t>2026-09-15 07:07 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="362">
+      <c r="A362" t="inlineStr">
+        <is>
+          <t>2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3484,7 +3491,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3650,7 +3657,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>
@@ -3786,7 +3793,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-15 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-17 07:06 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A362"/>
+  <dimension ref="A1:A363"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3468,6 +3468,13 @@
       <c r="A362" t="inlineStr">
         <is>
           <t>2026-09-16 07:07 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="363">
+      <c r="A363" t="inlineStr">
+        <is>
+          <t>2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3491,7 +3498,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3657,7 +3664,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>
@@ -3793,7 +3800,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-16 07:07 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-18 06:59 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A363"/>
+  <dimension ref="A1:A364"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3475,6 +3475,13 @@
       <c r="A363" t="inlineStr">
         <is>
           <t>2026-09-17 07:06 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="364">
+      <c r="A364" t="inlineStr">
+        <is>
+          <t>2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3498,7 +3505,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3664,7 +3671,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3800,7 +3807,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-17 07:06 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-19 06:57 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A364"/>
+  <dimension ref="A1:A365"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3482,6 +3482,13 @@
       <c r="A364" t="inlineStr">
         <is>
           <t>2026-09-18 06:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="365">
+      <c r="A365" t="inlineStr">
+        <is>
+          <t>2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3505,7 +3512,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3671,7 +3678,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3807,7 +3814,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-18 06:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-20 07:23 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A365"/>
+  <dimension ref="A1:A366"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3489,6 +3489,13 @@
       <c r="A365" t="inlineStr">
         <is>
           <t>2026-09-19 06:57 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="366">
+      <c r="A366" t="inlineStr">
+        <is>
+          <t>2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3512,7 +3519,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3678,7 +3685,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>
@@ -3814,7 +3821,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-19 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-21 07:33 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A366"/>
+  <dimension ref="A1:A367"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3496,6 +3496,13 @@
       <c r="A366" t="inlineStr">
         <is>
           <t>2026-09-20 07:23 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="367">
+      <c r="A367" t="inlineStr">
+        <is>
+          <t>2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -3519,7 +3526,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -3685,7 +3692,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>
@@ -3821,7 +3828,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-20 07:23 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-22 07:13 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A367"/>
+  <dimension ref="A1:A368"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3503,6 +3503,13 @@
       <c r="A367" t="inlineStr">
         <is>
           <t>2026-09-21 07:33 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="368">
+      <c r="A368" t="inlineStr">
+        <is>
+          <t>2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3526,7 +3533,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3692,7 +3699,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3828,7 +3835,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-21 07:33 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-23 07:14 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A368"/>
+  <dimension ref="A1:A369"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3510,6 +3510,13 @@
       <c r="A368" t="inlineStr">
         <is>
           <t>2026-09-22 07:13 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="369">
+      <c r="A369" t="inlineStr">
+        <is>
+          <t>2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3533,7 +3540,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3699,7 +3706,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3835,7 +3842,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-22 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-24 07:05 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A369"/>
+  <dimension ref="A1:A370"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3517,6 +3517,13 @@
       <c r="A369" t="inlineStr">
         <is>
           <t>2026-09-23 07:14 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="370">
+      <c r="A370" t="inlineStr">
+        <is>
+          <t>2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3540,7 +3547,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3706,7 +3713,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3842,7 +3849,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-23 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-25 07:03 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A370"/>
+  <dimension ref="A1:A371"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3524,6 +3524,13 @@
       <c r="A370" t="inlineStr">
         <is>
           <t>2026-09-24 07:05 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="371">
+      <c r="A371" t="inlineStr">
+        <is>
+          <t>2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>
@@ -3547,7 +3554,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>
@@ -3713,7 +3720,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>
@@ -3849,7 +3856,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-24 07:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-26 07:00 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A371"/>
+  <dimension ref="A1:A372"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3531,6 +3531,13 @@
       <c r="A371" t="inlineStr">
         <is>
           <t>2026-09-25 07:03 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="372">
+      <c r="A372" t="inlineStr">
+        <is>
+          <t>2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -3554,7 +3561,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -3720,7 +3727,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3863,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-25 07:03 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-27 07:31 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A372"/>
+  <dimension ref="A1:A373"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3538,6 +3538,13 @@
       <c r="A372" t="inlineStr">
         <is>
           <t>2026-09-26 07:00 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="373">
+      <c r="A373" t="inlineStr">
+        <is>
+          <t>2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3568,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3734,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3863,7 +3870,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-26 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-28 08:08 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A373"/>
+  <dimension ref="A1:A374"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3545,6 +3545,13 @@
       <c r="A373" t="inlineStr">
         <is>
           <t>2026-09-27 07:31 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="374">
+      <c r="A374" t="inlineStr">
+        <is>
+          <t>2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3568,7 +3575,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3734,7 +3741,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>
@@ -3870,7 +3877,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-27 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-29 07:49 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A374"/>
+  <dimension ref="A1:A375"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3552,6 +3552,13 @@
       <c r="A374" t="inlineStr">
         <is>
           <t>2026-09-28 08:08 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="375">
+      <c r="A375" t="inlineStr">
+        <is>
+          <t>2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>
@@ -3575,7 +3582,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>
@@ -3741,7 +3748,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>
@@ -3877,7 +3884,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-28 08:08 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-09-30 07:52 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A375"/>
+  <dimension ref="A1:A376"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3559,6 +3559,13 @@
       <c r="A375" t="inlineStr">
         <is>
           <t>2026-09-29 07:49 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="376">
+      <c r="A376" t="inlineStr">
+        <is>
+          <t>2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3582,7 +3589,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3748,7 +3755,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3884,7 +3891,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-29 07:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-01 08:14 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A376"/>
+  <dimension ref="A1:A377"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3566,6 +3566,13 @@
       <c r="A376" t="inlineStr">
         <is>
           <t>2026-09-30 07:52 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="377">
+      <c r="A377" t="inlineStr">
+        <is>
+          <t>2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3589,7 +3596,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3755,7 +3762,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3891,7 +3898,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-09-30 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-01 12:32 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A377"/>
+  <dimension ref="A1:A378"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3573,6 +3573,13 @@
       <c r="A377" t="inlineStr">
         <is>
           <t>2026-10-01 08:14 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="378">
+      <c r="A378" t="inlineStr">
+        <is>
+          <t>2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -3596,7 +3603,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -3762,7 +3769,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>
@@ -3898,7 +3905,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 08:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-02 07:52 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A378"/>
+  <dimension ref="A1:A379"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3580,6 +3580,13 @@
       <c r="A378" t="inlineStr">
         <is>
           <t>2026-10-01 12:32 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="379">
+      <c r="A379" t="inlineStr">
+        <is>
+          <t>2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3603,7 +3610,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3769,7 +3776,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3905,7 +3912,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-01 12:32 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-03 07:31 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A379"/>
+  <dimension ref="A1:A380"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3587,6 +3587,13 @@
       <c r="A379" t="inlineStr">
         <is>
           <t>2026-10-02 07:52 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="380">
+      <c r="A380" t="inlineStr">
+        <is>
+          <t>2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3610,7 +3617,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3776,7 +3783,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>
@@ -3912,7 +3919,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-02 07:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-04 07:42 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A380"/>
+  <dimension ref="A1:A381"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3594,6 +3594,13 @@
       <c r="A380" t="inlineStr">
         <is>
           <t>2026-10-03 07:31 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="381">
+      <c r="A381" t="inlineStr">
+        <is>
+          <t>2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3624,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>
@@ -3783,7 +3790,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>
@@ -3919,7 +3926,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-03 07:31 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-05 08:12 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A381"/>
+  <dimension ref="A1:A382"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3601,6 +3601,13 @@
       <c r="A381" t="inlineStr">
         <is>
           <t>2026-10-04 07:42 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="382">
+      <c r="A382" t="inlineStr">
+        <is>
+          <t>2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3624,7 +3631,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3790,7 +3797,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>
@@ -3926,7 +3933,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-04 07:42 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-06 08:29 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A382"/>
+  <dimension ref="A1:A383"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3608,6 +3608,13 @@
       <c r="A382" t="inlineStr">
         <is>
           <t>2026-10-05 08:12 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="383">
+      <c r="A383" t="inlineStr">
+        <is>
+          <t>2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3631,7 +3638,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3804,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3933,7 +3940,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-05 08:12 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-07 08:05 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A383"/>
+  <dimension ref="A1:A384"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3615,6 +3615,13 @@
       <c r="A383" t="inlineStr">
         <is>
           <t>2026-10-06 08:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="384">
+      <c r="A384" t="inlineStr">
+        <is>
+          <t>2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3638,7 +3645,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3804,7 +3811,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>
@@ -3940,7 +3947,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-06 08:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-08 08:21 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A384"/>
+  <dimension ref="A1:A385"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3622,6 +3622,13 @@
       <c r="A384" t="inlineStr">
         <is>
           <t>2026-10-07 08:05 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="385">
+      <c r="A385" t="inlineStr">
+        <is>
+          <t>2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3645,7 +3652,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3811,7 +3818,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3954,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-07 08:05 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-09 08:24 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A385"/>
+  <dimension ref="A1:A386"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3629,6 +3629,13 @@
       <c r="A385" t="inlineStr">
         <is>
           <t>2026-10-08 08:21 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="386">
+      <c r="A386" t="inlineStr">
+        <is>
+          <t>2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>
@@ -3652,7 +3659,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>
@@ -3818,7 +3825,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>
@@ -3954,7 +3961,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-08 08:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-10 08:01 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A386"/>
+  <dimension ref="A1:A387"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3636,6 +3636,13 @@
       <c r="A386" t="inlineStr">
         <is>
           <t>2026-10-09 08:24 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="387">
+      <c r="A387" t="inlineStr">
+        <is>
+          <t>2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3666,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>
@@ -3825,7 +3832,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>
@@ -3961,7 +3968,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-09 08:24 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-11 08:13 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A387"/>
+  <dimension ref="A1:A388"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3643,6 +3643,13 @@
       <c r="A387" t="inlineStr">
         <is>
           <t>2026-10-10 08:01 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="388">
+      <c r="A388" t="inlineStr">
+        <is>
+          <t>2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3666,7 +3673,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3832,7 +3839,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3968,7 +3975,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-10 08:01 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-12 08:30 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A388"/>
+  <dimension ref="A1:A389"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3650,6 +3650,13 @@
       <c r="A388" t="inlineStr">
         <is>
           <t>2026-10-11 08:13 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="389">
+      <c r="A389" t="inlineStr">
+        <is>
+          <t>2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>
@@ -3673,7 +3680,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>
@@ -3839,7 +3846,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>
@@ -3975,7 +3982,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-11 08:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-13 08:52 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A389"/>
+  <dimension ref="A1:A390"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3657,6 +3657,13 @@
       <c r="A389" t="inlineStr">
         <is>
           <t>2026-10-12 08:30 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="390">
+      <c r="A390" t="inlineStr">
+        <is>
+          <t>2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3680,7 +3687,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3846,7 +3853,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>
@@ -3982,7 +3989,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-12 08:30 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-14 07:02 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A390"/>
+  <dimension ref="A1:A391"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3664,6 +3664,13 @@
       <c r="A390" t="inlineStr">
         <is>
           <t>2026-10-13 08:52 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="391">
+      <c r="A391" t="inlineStr">
+        <is>
+          <t>2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>
@@ -3687,7 +3694,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>
@@ -3853,7 +3860,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>
@@ -3989,7 +3996,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-13 08:52 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-15 06:53 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A391"/>
+  <dimension ref="A1:A392"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3671,6 +3671,13 @@
       <c r="A391" t="inlineStr">
         <is>
           <t>2026-10-14 07:02 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="392">
+      <c r="A392" t="inlineStr">
+        <is>
+          <t>2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3694,7 +3701,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3860,7 +3867,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3996,7 +4003,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-14 07:02 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-16 06:40 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A392"/>
+  <dimension ref="A1:A393"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3678,6 +3678,13 @@
       <c r="A392" t="inlineStr">
         <is>
           <t>2026-10-15 06:53 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="393">
+      <c r="A393" t="inlineStr">
+        <is>
+          <t>2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3701,7 +3708,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>
@@ -3867,7 +3874,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>
@@ -4003,7 +4010,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-15 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-17 06:29 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A393"/>
+  <dimension ref="A1:A394"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3685,6 +3685,13 @@
       <c r="A393" t="inlineStr">
         <is>
           <t>2026-10-16 06:40 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="394">
+      <c r="A394" t="inlineStr">
+        <is>
+          <t>2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3708,7 +3715,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>
@@ -3874,7 +3881,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>
@@ -4010,7 +4017,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-16 06:40 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-18 06:54 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A394"/>
+  <dimension ref="A1:A395"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3692,6 +3692,13 @@
       <c r="A394" t="inlineStr">
         <is>
           <t>2026-10-17 06:29 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="395">
+      <c r="A395" t="inlineStr">
+        <is>
+          <t>2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3715,7 +3722,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>
@@ -3881,7 +3888,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>
@@ -4017,7 +4024,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-17 06:29 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-19 07:14 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A395"/>
+  <dimension ref="A1:A396"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3699,6 +3699,13 @@
       <c r="A395" t="inlineStr">
         <is>
           <t>2026-10-18 06:54 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="396">
+      <c r="A396" t="inlineStr">
+        <is>
+          <t>2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3722,7 +3729,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -3888,7 +3895,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>
@@ -4024,7 +4031,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-18 06:54 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-20 07:04 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A396"/>
+  <dimension ref="A1:A397"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3706,6 +3706,13 @@
       <c r="A396" t="inlineStr">
         <is>
           <t>2026-10-19 07:14 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="397">
+      <c r="A397" t="inlineStr">
+        <is>
+          <t>2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>
@@ -3729,7 +3736,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3902,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>
@@ -4031,7 +4038,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-19 07:14 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-21 06:57 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A397"/>
+  <dimension ref="A1:A398"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3713,6 +3713,13 @@
       <c r="A397" t="inlineStr">
         <is>
           <t>2026-10-20 07:04 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="398">
+      <c r="A398" t="inlineStr">
+        <is>
+          <t>2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3736,7 +3743,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3902,7 +3909,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4038,7 +4045,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-20 07:04 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-22 07:00 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A398"/>
+  <dimension ref="A1:A399"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3720,6 +3720,13 @@
       <c r="A398" t="inlineStr">
         <is>
           <t>2026-10-21 06:57 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="399">
+      <c r="A399" t="inlineStr">
+        <is>
+          <t>2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -3743,7 +3750,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -3909,7 +3916,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>
@@ -4045,7 +4052,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-21 06:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-23 06:53 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A399"/>
+  <dimension ref="A1:A400"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3727,6 +3727,13 @@
       <c r="A399" t="inlineStr">
         <is>
           <t>2026-10-22 07:00 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="400">
+      <c r="A400" t="inlineStr">
+        <is>
+          <t>2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3750,7 +3757,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -3916,7 +3923,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>
@@ -4052,7 +4059,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-22 07:00 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-24 06:49 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A400"/>
+  <dimension ref="A1:A401"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3734,6 +3734,13 @@
       <c r="A400" t="inlineStr">
         <is>
           <t>2026-10-23 06:53 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="401">
+      <c r="A401" t="inlineStr">
+        <is>
+          <t>2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>
@@ -3757,7 +3764,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>
@@ -3923,7 +3930,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>
@@ -4059,7 +4066,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-23 06:53 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-25 07:13 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A401"/>
+  <dimension ref="A1:A402"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3741,6 +3741,13 @@
       <c r="A401" t="inlineStr">
         <is>
           <t>2026-10-24 06:49 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="402">
+      <c r="A402" t="inlineStr">
+        <is>
+          <t>2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3764,7 +3771,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3930,7 +3937,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4066,7 +4073,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-24 06:49 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-26 07:21 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A402"/>
+  <dimension ref="A1:A403"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3748,6 +3748,13 @@
       <c r="A402" t="inlineStr">
         <is>
           <t>2026-10-25 07:13 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="403">
+      <c r="A403" t="inlineStr">
+        <is>
+          <t>2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3771,7 +3778,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>
@@ -3937,7 +3944,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>
@@ -4073,7 +4080,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-25 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-27 07:13 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A403"/>
+  <dimension ref="A1:A404"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3755,6 +3755,13 @@
       <c r="A403" t="inlineStr">
         <is>
           <t>2026-10-26 07:21 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="404">
+      <c r="A404" t="inlineStr">
+        <is>
+          <t>2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3778,7 +3785,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -3944,7 +3951,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>
@@ -4080,7 +4087,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-26 07:21 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-28 07:51 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A404"/>
+  <dimension ref="A1:A405"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3762,6 +3762,13 @@
       <c r="A404" t="inlineStr">
         <is>
           <t>2026-10-27 07:13 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="405">
+      <c r="A405" t="inlineStr">
+        <is>
+          <t>2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3785,7 +3792,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>
@@ -3951,7 +3958,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>
@@ -4087,7 +4094,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-27 07:13 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-29 07:57 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A405"/>
+  <dimension ref="A1:A406"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3769,6 +3769,13 @@
       <c r="A405" t="inlineStr">
         <is>
           <t>2026-10-28 07:51 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="406">
+      <c r="A406" t="inlineStr">
+        <is>
+          <t>2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3792,7 +3799,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -3958,7 +3965,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>
@@ -4094,7 +4101,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-28 07:51 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-30 07:59 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A406"/>
+  <dimension ref="A1:A407"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3776,6 +3776,13 @@
       <c r="A406" t="inlineStr">
         <is>
           <t>2026-10-29 07:57 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="407">
+      <c r="A407" t="inlineStr">
+        <is>
+          <t>2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3799,7 +3806,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>
@@ -3965,7 +3972,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>
@@ -4101,7 +4108,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-29 07:57 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
ci: refresh reports & README last-run summary (2026-10-31 07:56 UTC)
</commit_message>
<xml_diff>
--- a/04_Excel/01_Data_Overview.xlsx
+++ b/04_Excel/01_Data_Overview.xlsx
@@ -515,7 +515,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>
@@ -707,7 +707,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>
@@ -934,7 +934,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A407"/>
+  <dimension ref="A1:A408"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3783,6 +3783,13 @@
       <c r="A407" t="inlineStr">
         <is>
           <t>2026-10-30 07:59 UTC</t>
+        </is>
+      </c>
+    </row>
+    <row r="408">
+      <c r="A408" t="inlineStr">
+        <is>
+          <t>2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3806,7 +3813,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>
@@ -3972,7 +3979,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>
@@ -4108,7 +4115,7 @@
     <row r="1">
       <c r="A1" s="4" t="inlineStr">
         <is>
-          <t>Last Refreshed (UTC): 2026-10-30 07:59 UTC</t>
+          <t>Last Refreshed (UTC): 2026-10-31 07:56 UTC</t>
         </is>
       </c>
     </row>

</xml_diff>